<commit_message>
Add Language_Control sheet per RFC-002 / Decision-018
Adds a new Language_Control sheet to templates/Character_Profile_Template_v1.0.xlsx
with Description_CN (required), Description_EN, Prompt_CN, and Prompt_EN,
per RFC0002 Section 4.1 and Decision-018's Language Ownership Rule.
Kept as a separate sheet rather than extending Prompt_Control, since language
is a cross-cutting governance layer rather than generation-only control.

No Caption fields added (out of scope for Character Profile per RFC0002
Section 4.2/4.3). schemas/ and generators/ untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Character_Profile_Template_v1.0.xlsx
+++ b/templates/Character_Profile_Template_v1.0.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Costume_Identity" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Behavior_Identity" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Prompt_Control" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Language_Control" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2179,4 +2180,160 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field_Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Data_Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Description_CN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Canonical human-authored historical description in Chinese. This is the authoritative source of historical meaning (Decision-018).</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>萧绰，辽朝皇太后，临朝摄政。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Description_EN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Optional English translation of Description_CN for human reference. Derived from the Chinese source; does not replace it.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Xiao Chuo, Liao Dynasty Empress Dowager, acted as regent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Prompt_CN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Optional Chinese-language generation prompt fragment derived from this character profile.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>萧绰，辽朝，皇太后，站立，目视前方</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Prompt_EN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>English prompt is a model adaptation layer and cannot override the Chinese semantic source (Description_CN, Prompt_CN).</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Xiao Chuo, Liao, Empress Dowager, standing, looking forward</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>